<commit_message>
circo : l'annexe VI, le partage de 1986, et Paris jusqu'à 1815
- controle_annexe_vi.py et annexe_vi_villes_divisees.csv confrontent
  l'atlas de Gaudillère au ministère, source indépendante contre source
  officielle.
- circo_1986_partage.csv et son correctif : les cantons que le décret
  laisse indéterminés, tranchés par l'atlas.
- remonte_1815.py, paris_quartiers_1815.py, paris_circo_1815 :
  la base parisienne remonte à 1815, sur la trame des 80 quartiers.
</commit_message>
<xml_diff>
--- a/circo/paris_decoupage.xlsx
+++ b/circo/paris_decoupage.xlsx
@@ -151,7 +151,7 @@
     <t xml:space="preserve">porte saint martin, saint martin des champs, temple</t>
   </si>
   <si>
-    <t xml:space="preserve">popincourt, mont de piétémarais, marché saint-jean, faubourg saint-antoine, quinze-vingts</t>
+    <t xml:space="preserve">popincourt, mont de piété, marais, marché saint-jean, faubourg saint-antoine, quinze-vingts</t>
   </si>
   <si>
     <t xml:space="preserve">saint-jacques, observatoire, jardin-des-plantes, saint-marcel, sorbonne, ile saint louis, arsenal</t>
@@ -987,9 +987,9 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E423"/>
-  <sheetFormatPr defaultColWidth="10.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.54296875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="23.69"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="117.31"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="24.43"/>
   </cols>
   <sheetData>

</xml_diff>